<commit_message>
added datatable and fixed some data points
</commit_message>
<xml_diff>
--- a/data_points.xlsx
+++ b/data_points.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="63">
   <si>
     <t xml:space="preserve">Händelse</t>
   </si>
@@ -181,10 +181,10 @@
     <t xml:space="preserve">Middag med Lotta, Robban och Lovisas pappa</t>
   </si>
   <si>
-    <t xml:space="preserve">59.31333442537845</t>
-  </si>
-  <si>
-    <t xml:space="preserve">159.313334425378458.0934103236601</t>
+    <t xml:space="preserve">59.31311709100336</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.09491759452525</t>
   </si>
   <si>
     <t xml:space="preserve">2026.V.20</t>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t xml:space="preserve">18.058712068969136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.26</t>
   </si>
 </sst>
 </file>
@@ -215,7 +218,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,12 +248,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="5.5"/>
@@ -302,7 +299,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -319,11 +316,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -772,13 +765,13 @@
       <c r="A16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -786,16 +779,16 @@
       <c r="A17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>56</v>
       </c>
     </row>
@@ -817,15 +810,18 @@
       <c r="A19" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>61</v>
       </c>
+      <c r="D19" s="0" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="5"/>
+      <c r="G28" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
ordered data points again and fixed column widths
</commit_message>
<xml_diff>
--- a/data_points.xlsx
+++ b/data_points.xlsx
@@ -76,6 +76,18 @@
     <t xml:space="preserve">2026.III.06</t>
   </si>
   <si>
+    <t xml:space="preserve">Första nära</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tillsammans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.08</t>
+  </si>
+  <si>
     <t xml:space="preserve">Första översovning hos Lovisa</t>
   </si>
   <si>
@@ -88,40 +100,28 @@
     <t xml:space="preserve">2026.III.10</t>
   </si>
   <si>
-    <t xml:space="preserve">Tillsammans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026.III.08</t>
+    <t xml:space="preserve">Första biodejten (Doktor Glas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59.33442658656568</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.062658380025532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">William träffar Lovisas pappa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.19</t>
   </si>
   <si>
     <t xml:space="preserve">Första jag älskar dig</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Första biodejten (Doktor Glas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59.33442658656568</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.062658380025532</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026.III.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Första nära</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026.III.07</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första hela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">William träffar Lovisas pappa</t>
   </si>
   <si>
     <t xml:space="preserve">Första PONG Buffé-dejten</t>
@@ -510,7 +510,7 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.08"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -595,19 +595,18 @@
         <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>13</v>
@@ -616,19 +615,19 @@
         <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>25</v>
@@ -655,10 +654,10 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>31</v>
@@ -669,27 +668,28 @@
         <v>32</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>25</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -797,6 +797,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="0"/>
+      <c r="D20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0"/>
+      <c r="D21" s="0"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G28" s="4"/>

</xml_diff>

<commit_message>
added javascript addition in order to center map on selected events
</commit_message>
<xml_diff>
--- a/data_points.xlsx
+++ b/data_points.xlsx
@@ -25,30 +25,30 @@
     <t xml:space="preserve">Händelse</t>
   </si>
   <si>
-    <t xml:space="preserve">Lattitude</t>
+    <t xml:space="preserve">Datum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latitude</t>
   </si>
   <si>
     <t xml:space="preserve">Longitude</t>
   </si>
   <si>
-    <t xml:space="preserve">Datum</t>
-  </si>
-  <si>
     <t xml:space="preserve">Typ</t>
   </si>
   <si>
     <t xml:space="preserve">Första dejten</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.II.28</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.335921109724076</t>
   </si>
   <si>
     <t xml:space="preserve">18.033817926639617</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.II.28</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första kyssen</t>
   </si>
   <si>
@@ -61,15 +61,15 @@
     <t xml:space="preserve">Första hemmadjeten hos William</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.III.03</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.762464999923004</t>
   </si>
   <si>
     <t xml:space="preserve">18.692603259162077</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.03</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första översovning hos William</t>
   </si>
   <si>
@@ -91,39 +91,39 @@
     <t xml:space="preserve">Första norrtäljebussen tillsammans</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.III.09</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.759610766683764</t>
   </si>
   <si>
     <t xml:space="preserve">18.699794522093505</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.09</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första översovning hos Lovisa</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.III.10</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.35976722179485</t>
   </si>
   <si>
     <t xml:space="preserve">17.838707815604636</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första biodejten (Doktor Glas)</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.III.14</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.33442658656568</t>
   </si>
   <si>
     <t xml:space="preserve">18.062658380025532</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.14</t>
-  </si>
-  <si>
     <t xml:space="preserve">William träffar Lovisas pappa</t>
   </si>
   <si>
@@ -139,51 +139,51 @@
     <t xml:space="preserve">Första PONG Buffé-dejten</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.III.26</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.33643177461977</t>
   </si>
   <si>
     <t xml:space="preserve">18.058712068969136</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.III.26</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lovisa träffar Williams pappa och syskon</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.IV.04</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.33343415093351</t>
   </si>
   <si>
     <t xml:space="preserve">18.090619846453873</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.IV.04</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lovisa är på Williams jobb för första gången</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.IV.08</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.36835226081049</t>
   </si>
   <si>
     <t xml:space="preserve">18.054884785647378</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.IV.08</t>
-  </si>
-  <si>
     <t xml:space="preserve">William träffar Lovisas mormor</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.IV.12</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.361898035202984</t>
   </si>
   <si>
     <t xml:space="preserve">17.839487795478654</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.IV.12</t>
-  </si>
-  <si>
     <t xml:space="preserve">Såg första David Lynch-filmen (Blue Velvet)</t>
   </si>
   <si>
@@ -193,15 +193,15 @@
     <t xml:space="preserve">Första översovning på landet</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.IV.30</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.992206824075666</t>
   </si>
   <si>
     <t xml:space="preserve">18.770247299844495</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.IV.30</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första landet</t>
   </si>
   <si>
@@ -211,64 +211,64 @@
     <t xml:space="preserve">William är med Lovisa på Makeriet</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.V.14</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.31065897460733</t>
   </si>
   <si>
     <t xml:space="preserve">18.076689568967716</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.V.14</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lovisa träffar Williams farfar och pappas sida av släkten</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.V.17</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.510705896222426</t>
   </si>
   <si>
     <t xml:space="preserve">17.760380450066414</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.V.17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Middag med Lotta, Robban och Lovisas pappa</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.V.20</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.31311709100336</t>
   </si>
   <si>
     <t xml:space="preserve">18.09491759452525</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.V.20</t>
-  </si>
-  <si>
     <t xml:space="preserve">oklar plats</t>
   </si>
   <si>
     <t xml:space="preserve">William följer med till Lovisas mammas grav för första gången</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.V.21</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.364929230932745</t>
   </si>
   <si>
     <t xml:space="preserve">17.826940410064022</t>
   </si>
   <si>
-    <t xml:space="preserve">2026.V.21</t>
-  </si>
-  <si>
     <t xml:space="preserve">Första Hemmakväll-dejten</t>
   </si>
   <si>
+    <t xml:space="preserve">2026.V.24</t>
+  </si>
+  <si>
     <t xml:space="preserve">59.759613992355014</t>
   </si>
   <si>
     <t xml:space="preserve">18.703543727641744</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026.V.24</t>
   </si>
   <si>
     <t xml:space="preserve">Översovning varje dag i en månad</t>
@@ -582,7 +582,7 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.08"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -601,18 +601,19 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="1"/>
@@ -621,14 +622,14 @@
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="E3" s="1"/>
     </row>
@@ -636,13 +637,13 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="1"/>
@@ -651,14 +652,14 @@
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
+      <c r="B5" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>17</v>
+      <c r="D5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="E5" s="1"/>
     </row>
@@ -666,28 +667,28 @@
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>13</v>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>19</v>
+      <c r="D6" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="E7" s="1"/>
     </row>
@@ -698,10 +699,10 @@
       <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="3" t="s">
         <v>25</v>
       </c>
     </row>
@@ -709,13 +710,13 @@
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="1"/>
@@ -724,13 +725,13 @@
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E10" s="1"/>
@@ -739,28 +740,28 @@
       <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>27</v>
+      <c r="B11" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>35</v>
+      <c r="D11" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>27</v>
+      <c r="B12" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>35</v>
+      <c r="D12" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="E12" s="1"/>
     </row>
@@ -768,27 +769,27 @@
       <c r="A13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>27</v>
+      <c r="B13" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>35</v>
+      <c r="D13" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="3" t="s">
         <v>41</v>
       </c>
     </row>
@@ -796,13 +797,13 @@
       <c r="A15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -810,13 +811,13 @@
       <c r="A16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -824,42 +825,42 @@
       <c r="A17" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>27</v>
+      <c r="B18" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="0" t="s">
-        <v>55</v>
+      <c r="D18" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E19" s="1"/>
@@ -868,27 +869,27 @@
       <c r="A20" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>57</v>
+      <c r="B20" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>61</v>
+      <c r="D20" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="3" t="s">
         <v>65</v>
       </c>
     </row>
@@ -896,13 +897,13 @@
       <c r="A22" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="3" t="s">
         <v>69</v>
       </c>
     </row>
@@ -910,13 +911,13 @@
       <c r="A23" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>71</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E23" s="1" t="s">
@@ -927,13 +928,13 @@
       <c r="A24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>76</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="3" t="s">
         <v>78</v>
       </c>
     </row>
@@ -941,13 +942,13 @@
       <c r="A25" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="3" t="s">
         <v>82</v>
       </c>
     </row>
@@ -955,14 +956,14 @@
       <c r="A26" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>13</v>
+      <c r="B26" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>84</v>
+      <c r="D26" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
added datapoints and updated formatting
</commit_message>
<xml_diff>
--- a/data_points.xlsx
+++ b/data_points.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="97">
   <si>
     <t xml:space="preserve">Händelse</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Typ</t>
   </si>
   <si>
-    <t xml:space="preserve">Första dejten</t>
+    <t xml:space="preserve">Första dejten (Biljardpalatset)</t>
   </si>
   <si>
     <t xml:space="preserve">2026.II.28</t>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">18.062658380025532</t>
   </si>
   <si>
-    <t xml:space="preserve">Första fikadejten</t>
+    <t xml:space="preserve">Första fikadejten (Espresso House)</t>
   </si>
   <si>
     <t xml:space="preserve">2026.III.18</t>
@@ -160,6 +160,12 @@
     <t xml:space="preserve">18.058712068969136</t>
   </si>
   <si>
+    <t xml:space="preserve">Firar 1 månad tillsammans (trött morgon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.III.28</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lovisa träffar Williams pappa och syskon</t>
   </si>
   <si>
@@ -202,6 +208,12 @@
     <t xml:space="preserve">2026.IV.18</t>
   </si>
   <si>
+    <t xml:space="preserve">Firar 2 månader tillsammans (lyxbrunch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.IV.28</t>
+  </si>
+  <si>
     <t xml:space="preserve">Första översovning på landet</t>
   </si>
   <si>
@@ -287,6 +299,18 @@
   </si>
   <si>
     <t xml:space="preserve">2026.V.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firar 3 månader tillsammans (bio: Project Hail Mary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.V.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59.37149195601381</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.003406770817737</t>
   </si>
 </sst>
 </file>
@@ -296,7 +320,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -326,12 +350,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="5.5"/>
@@ -383,7 +401,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -400,11 +418,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -600,7 +614,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.19"/>
@@ -759,16 +773,16 @@
       <c r="E10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>37</v>
       </c>
     </row>
@@ -837,54 +851,54 @@
         <v>47</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="D17" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="D18" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="D19" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
@@ -894,116 +908,156 @@
         <v>61</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="C21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="C22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="D22" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>69</v>
-      </c>
+      <c r="E22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C28" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="5"/>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G30" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>